<commit_message>
Rename instruments to CPS XXXX / CPG XXXX
The supplied draft AI standard is already titled CPS XXX, and this
package's M34 boundary rule exists to separate the two instruments,
so a four-X placeholder avoids an ambiguous cross-reference.

Also adds OSFI E-23 section A.4's six stakeholder roles to the
principles register and to M07's principle mapping.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9tVmgcRH2aPufRoj4ddoe
</commit_message>
<xml_diff>
--- a/MRM_Regulatory_Comparison_and_Improvement_Assessment.xlsx
+++ b/MRM_Regulatory_Comparison_and_Improvement_Assessment.xlsx
@@ -526,7 +526,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Adopt a broad function-based definition of a model and of model risk on a cross-industry basis, with an express obligation to identify and control quantitative tools falling outside it. Do not follow the April 2026 United States narrowing, which would exclude actuarial and unit pricing calculations.</t>
         </r>
       </text>
@@ -539,7 +539,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 State enterprise-wide application expressly and confirm that accountability is retained where a model is supplied or operated by another party.</t>
         </r>
       </text>
@@ -552,7 +552,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require a complete, current, controlled enterprise inventory including embedded, third-party and recently decommissioned models, with minimum fields specified.</t>
         </r>
       </text>
@@ -565,7 +565,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require a documented tiering methodology using quantitative and qualitative factors that demonstrably drives validation, monitoring and approval intensity.</t>
         </r>
       </text>
@@ -578,7 +578,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require Board approval of the model risk framework and appetite, supported by aggregate, decision-useful reporting rather than model counts.</t>
         </r>
       </text>
@@ -591,7 +591,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require a named senior executive accountable for the framework, plus a named owner for each model, and settle the interaction with the accountability regime.</t>
         </r>
       </text>
@@ -604,7 +604,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require an appetite for model risk expressed so that it can be measured, with limits, thresholds and escalation triggers.</t>
         </r>
       </text>
@@ -617,7 +617,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require documented development standards, conceptual soundness, consideration of alternatives and recording of limitations across all material models.</t>
         </r>
       </text>
@@ -630,7 +630,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require model data to be assessed for appropriateness as well as quality, with lineage to source and documented treatment of proxies and synthetic data.</t>
         </r>
       </text>
@@ -643,7 +643,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Adopt the reconstruction test: documentation sufficient for an independent competent person to reproduce material results.</t>
         </r>
       </text>
@@ -656,7 +656,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Establish an explicit gate: a model must not be used for a material purpose until tested and residual limitations accepted.</t>
         </r>
       </text>
@@ -669,7 +669,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require independent validation for material models, structured around conceptual soundness, ongoing monitoring and outcomes analysis, at an intensity set by tier.</t>
         </r>
       </text>
@@ -682,7 +682,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require effective challenge expressly, and expect entities to assess whether it is operating through finding closure routes and severity migration.</t>
         </r>
       </text>
@@ -695,7 +695,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require version-specific approval for a defined purpose and conditions, recording limits, thresholds, accepted limitations and review date.</t>
         </r>
       </text>
@@ -708,7 +708,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require pre-production verification against the approved model and re-verification after material infrastructure or pipeline change.</t>
         </r>
       </text>
@@ -721,7 +721,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require materiality assessment of changes individually and cumulatively, and treat provider-initiated change as an entity change event.</t>
         </r>
       </text>
@@ -734,7 +734,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require use within approved purpose and conditions, and require limitations to be communicated to users rather than merely recorded.</t>
         </r>
       </text>
@@ -747,7 +747,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require governance of the basis, quantification, approval, duration and removal of overlays, and aggregate reporting of them.</t>
         </r>
       </text>
@@ -760,7 +760,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require monitoring at tier-based frequency with pre-set thresholds linked to investigation, restriction, revalidation or withdrawal.</t>
         </r>
       </text>
@@ -773,7 +773,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require recorded limitations, specific compensating controls, tracked remediation and escalation of overdue material findings.</t>
         </r>
       </text>
@@ -786,7 +786,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require managed decommissioning covering downstream models, outputs still in force, records and data disposition.</t>
         </r>
       </text>
@@ -799,7 +799,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Apply the full framework to third-party models, require usable information rights without mandating source-code access, and require compensating controls where information is unavailable.</t>
         </r>
       </text>
@@ -812,7 +812,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require entity-level concentration assessment and support sector-wide monitoring of common model and data dependencies.</t>
         </r>
       </text>
@@ -825,7 +825,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Bring AI models within the model risk framework as a model class, with an explicit boundary rule against the AI risk instrument so nothing falls between.</t>
         </r>
       </text>
@@ -838,8 +838,8 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
-Preserve the capital standards unchanged and position CPS 240 to sit alongside them, with the more specific requirement prevailing.</t>
+          <t xml:space="preserve">Expected position after CPS XXXX:
+Preserve the capital standards unchanged and position CPS XXXX to sit alongside them, with the more specific requirement prevailing.</t>
         </r>
       </text>
     </comment>
@@ -851,7 +851,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Bring valuation and expected credit loss models expressly within scope and require independent price verification as a control distinct from validation.</t>
         </r>
       </text>
@@ -864,7 +864,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require insurers to map which validation elements the actuarial control cycle discharges and which need separate work.</t>
         </r>
       </text>
@@ -877,7 +877,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Name the RSE model classes expressly. Scored against the cross-industry benchmark rather than a comparator, because none exists.</t>
         </r>
       </text>
@@ -890,7 +890,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Bring stress testing, scenario and capital planning models within scope, with explicit treatment of assumption governance and of uncertainty disclosure.</t>
         </r>
       </text>
@@ -903,7 +903,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require aggregate assessment and consideration in internal capital assessment, permitting qualitative measures where quantification is not yet feasible.</t>
         </r>
       </text>
@@ -916,7 +916,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Specify reconstructability for material models, with retention aligned to the period over which the decisions informed remain material.</t>
         </r>
       </text>
@@ -929,7 +929,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Require periodic independent assessment of framework design and operating effectiveness, including the effectiveness of validation and challenge.</t>
         </r>
       </text>
@@ -942,7 +942,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Expected position after CPS 240:
+          <t xml:space="preserve">Expected position after CPS XXXX:
 Cross-reference existing CPS 230 and CPS 234 timeframes rather than create a conflicting deadline, and expect early engagement on material model weakness.</t>
         </r>
       </text>
@@ -969,7 +969,7 @@
     <t xml:space="preserve">Package status</t>
   </si>
   <si>
-    <t xml:space="preserve">POLICY DEVELOPMENT DRAFT — NOT IN FORCE. This workbook, the draft CPS 240 and the draft CPG 240 are policy-development artefacts with no legal effect.</t>
+    <t xml:space="preserve">POLICY DEVELOPMENT DRAFT — NOT IN FORCE. This workbook, the draft CPS XXXX and the draft CPG XXXX are policy-development artefacts with no legal effect.</t>
   </si>
   <si>
     <t xml:space="preserve">As-of date</t>
@@ -1050,7 +1050,7 @@
     <t xml:space="preserve">Draft mandatory requirements</t>
   </si>
   <si>
-    <t xml:space="preserve">Bold mandatory paragraphs in draft CPS 240.</t>
+    <t xml:space="preserve">Bold mandatory paragraphs in draft CPS XXXX.</t>
   </si>
   <si>
     <t xml:space="preserve">Requirements that are policy choices</t>
@@ -1065,7 +1065,7 @@
     <t xml:space="preserve">Carry an express legal-drafting reservation.</t>
   </si>
   <si>
-    <t xml:space="preserve">Guidance paragraphs in draft CPG 240</t>
+    <t xml:space="preserve">Guidance paragraphs in draft CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Every requirement has at least one supporting guidance paragraph.</t>
@@ -1083,10 +1083,10 @@
     <t xml:space="preserve">Weighted mean across all domains of the framework as it stands today.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mean expected score after CPS 240</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expected position once CPS 240 and CPG 240 are in force.</t>
+    <t xml:space="preserve">Mean expected score after CPS XXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected position once CPS XXXX and CPG XXXX are in force.</t>
   </si>
   <si>
     <t xml:space="preserve">Critical priority gaps</t>
@@ -1305,7 +1305,7 @@
     <t xml:space="preserve">Gap × domain weight. This is what drives the priority band.</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected score after CPS 240</t>
+    <t xml:space="preserve">Expected score after CPS XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Assessed position once the draft standard and guide are in force, on the same 0–5 scale. The difference from the current score is the value the instrument is expected to add.</t>
@@ -1470,7 +1470,7 @@
     <t xml:space="preserve">Worked example</t>
   </si>
   <si>
-    <t xml:space="preserve">'Definition of a model and of model risk' scores 1, 1, 2 and 1 on coverage, specificity, enforceability and alignment, giving a domain score of 1.25. The strongest comparator is PRA / OSFI at 5. The gap is 5 − 1.25 = 3.75. The domain weight is 1.5, so the weighted gap is 5.62, which falls in the Critical band. After CPS 240 the expected score is 4.5.</t>
+    <t xml:space="preserve">'Definition of a model and of model risk' scores 1, 1, 2 and 1 on coverage, specificity, enforceability and alignment, giving a domain score of 1.25. The strongest comparator is PRA / OSFI at 5. The gap is 5 − 1.25 = 3.75. The domain weight is 1.5, so the weighted gap is 5.62, which falls in the Critical band. After CPS XXXX the expected score is 4.5.</t>
   </si>
   <si>
     <t xml:space="preserve">Limitations of this scoring</t>
@@ -1485,7 +1485,7 @@
     <t xml:space="preserve">• Legal status is scored as it stands in the home jurisdiction. It does not imply that any overseas instrument has effect in Australia.</t>
   </si>
   <si>
-    <t xml:space="preserve">• The expected post-CPS 240 score assumes the draft is issued substantially as drafted and is implemented as intended. It is a design expectation, not an outcome.</t>
+    <t xml:space="preserve">• The expected post-CPS XXXX score assumes the draft is issued substantially as drafted and is implemented as intended. It is a design expectation, not an outcome.</t>
   </si>
   <si>
     <t xml:space="preserve">Gap assessment — current Australian framework against strongest comparator</t>
@@ -1503,13 +1503,13 @@
     <t xml:space="preserve">Priority</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected after CPS 240</t>
+    <t xml:space="preserve">Expected after CPS XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Uplift</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 requirements</t>
+    <t xml:space="preserve">CPS XXXX requirements</t>
   </si>
   <si>
     <t xml:space="preserve">Source IDs</t>
@@ -1980,7 +1980,7 @@
     <t xml:space="preserve">This is the strongest part of the Australian framework. The residual gap is the absence of a general model risk discipline around the capital model estate, and less developed guidance on model change than the ECB provides.</t>
   </si>
   <si>
-    <t xml:space="preserve">Preserve the capital standards unchanged and position CPS 240 to sit alongside them, with the more specific requirement prevailing.</t>
+    <t xml:space="preserve">Preserve the capital standards unchanged and position CPS XXXX to sit alongside them, with the more specific requirement prevailing.</t>
   </si>
   <si>
     <t xml:space="preserve">The Appointed Actuary framework is a genuine strength but was not designed as model risk management. Implementation verification and data quality assessment are not reliably covered.</t>
@@ -2028,7 +2028,7 @@
     <t xml:space="preserve">FSB</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposed CPS 240 position</t>
+    <t xml:space="preserve">Proposed CPS XXXX position</t>
   </si>
   <si>
     <t xml:space="preserve">Legal character of the framework</t>
@@ -3240,7 +3240,7 @@
     <t xml:space="preserve">Prudential Standard SPS 515 Strategic Planning and Member Outcomes</t>
   </si>
   <si>
-    <t xml:space="preserve">Draft CPS 240 requirements register</t>
+    <t xml:space="preserve">Draft CPS XXXX requirements register</t>
   </si>
   <si>
     <t xml:space="preserve">POLICY DEVELOPMENT DRAFT — NOT IN FORCE | Mandatory wording appears in bold in the Word standard; this sheet records provenance and rationale.</t>
@@ -3276,7 +3276,7 @@
     <t xml:space="preserve">International principle</t>
   </si>
   <si>
-    <t xml:space="preserve">CPG 240 paragraphs</t>
+    <t xml:space="preserve">CPG XXXX paragraphs</t>
   </si>
   <si>
     <t xml:space="preserve">Part A — Application and interpretation</t>
@@ -3426,7 +3426,7 @@
     <t xml:space="preserve">Role definition with named model owners is explicit in the US, Canadian and ECB material.</t>
   </si>
   <si>
-    <t xml:space="preserve">US interagency guidance 2026 §VI roles; OSFI E-23 roles and responsibilities; ECB internal governance</t>
+    <t xml:space="preserve">US interagency guidance 2026 §VI (roles and responsibilities); OSFI E-23 (2027) §A.4, defining Model Owner, Model Developer, Model Reviewer, Model Approver, Model User and Model Stakeholder; ECB guide §5</t>
   </si>
   <si>
     <t xml:space="preserve">32–33</t>
@@ -4203,7 +4203,7 @@
     <t xml:space="preserve">Diverges</t>
   </si>
   <si>
-    <t xml:space="preserve">US-MRM-2026, PRA-SS1-23, OSFI-E23  |  OCC/Fed: The April 2026 guidance narrows the definition to complex methods and excludes spreadsheet arithmetic, deterministic rules and generative and agentic AI. CPS 240 does not follow.</t>
+    <t xml:space="preserve">US-MRM-2026, PRA-SS1-23, OSFI-E23  |  OCC/Fed: The April 2026 guidance narrows the definition to complex methods and excludes spreadsheet arithmetic, deterministic rules and generative and agentic AI. CPS XXXX does not follow.</t>
   </si>
   <si>
     <t xml:space="preserve">PRA-SS1-23, OSFI-E23  |  OCC/Fed: Expressly excludes such tools from the model definition and states no control obligation for them.</t>
@@ -4251,7 +4251,7 @@
     <t xml:space="preserve">POLICY DEVELOPMENT DRAFT — NOT IN FORCE | Every numbered paragraph of the draft practice guide, and the requirement it supports.</t>
   </si>
   <si>
-    <t xml:space="preserve">CPG 240 paragraph</t>
+    <t xml:space="preserve">CPG XXXX paragraph</t>
   </si>
   <si>
     <t xml:space="preserve">Chapter</t>
@@ -4260,7 +4260,7 @@
     <t xml:space="preserve">Guidance text</t>
   </si>
   <si>
-    <t xml:space="preserve">Supports CPS 240</t>
+    <t xml:space="preserve">Supports CPS XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Source attribution</t>
@@ -4272,13 +4272,13 @@
     <t xml:space="preserve">Introduction</t>
   </si>
   <si>
-    <t xml:space="preserve">This guide is structured to follow CPS 240. Each chapter opens with the requirements it supports, so that a reader working from the standard can find the corresponding guidance, and a reader working from the guidance can identify the obligation it explains.</t>
+    <t xml:space="preserve">This guide is structured to follow CPS XXXX. Each chapter opens with the requirements it supports, so that a reader working from the standard can find the corresponding guidance, and a reader working from the guidance can identify the obligation it explains.</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">Guidance in this guide is drawn from Australian prudential requirements and from the model risk frameworks of comparable authorities. International sources are labelled by legal status: [B] binding in its home jurisdiction, [SE] supervisory expectation, [G] guidance, [PB] proposed or consultative, and [A] analytical or advisory. An overseas instrument is not binding in Australia whatever its status at home, and is used here only to inform expectations under CPS 240.</t>
+    <t xml:space="preserve">Guidance in this guide is drawn from Australian prudential requirements and from the model risk frameworks of comparable authorities. International sources are labelled by legal status: [B] binding in its home jurisdiction, [SE] supervisory expectation, [G] guidance, [PB] proposed or consultative, and [A] analytical or advisory. An overseas instrument is not binding in Australia whatever its status at home, and is used here only to inform expectations under CPS XXXX.</t>
   </si>
   <si>
     <t xml:space="preserve">Status classification follows Annex D of this guide and the source register in the accompanying assessment workbook.</t>
@@ -4287,7 +4287,7 @@
     <t xml:space="preserve">APRA expects this guide to be applied proportionately. An entity with a small number of vendor models and one with several hundred internally developed models across banking, insurance and superannuation businesses face the same obligations but will meet them very differently.</t>
   </si>
   <si>
-    <t xml:space="preserve">This guide does not create obligations, does not vary CPS 240, and does not limit APRA's discretion in supervising an entity. Where this guide and CPS 240 appear to differ, CPS 240 prevails.</t>
+    <t xml:space="preserve">This guide does not create obligations, does not vary CPS XXXX, and does not limit APRA's discretion in supervising an entity. Where this guide and CPS XXXX appear to differ, CPS XXXX prevails.</t>
   </si>
   <si>
     <t xml:space="preserve">Regulated entities have increased their reliance on models faster than they have increased their capacity to govern them. Models now determine capital, provisions, valuations, insurance liabilities, unit prices, credit decisions, fraud interventions and member outcomes. The consequence of a model being wrong has grown with the consequence of the decisions it drives.</t>
@@ -4314,7 +4314,7 @@
     <t xml:space="preserve">Source: PRA SS1/23 Principle 1.1 Model definition [SE]. OSFI Guideline E-23 (2027), key terms [SE]. The three-component description originated in the 2011 United States interagency guidance, which was rescinded on 17 April 2026; the description remains analytically useful and is retained here on that basis rather than as a current citation.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verification: the United States interagency guidance was revised on 17 April 2026 (SR 26-2, OCC Bulletin 2026-13, FDIC FIL-15-2026), rescinding the 2011 guidance. The 2026 definition is narrower — a 'complex' quantitative method applying statistical, economic or financial theories, expressly excluding simple arithmetic such as spreadsheet calculations and deterministic rule-based processes, and expressly excluding generative and agentic AI. CPS 240 does not adopt that narrowing, for the reasons given in the standard. The divergence is deliberate.</t>
+    <t xml:space="preserve">Verification: the United States interagency guidance was revised on 17 April 2026 (SR 26-2, OCC Bulletin 2026-13, FDIC FIL-15-2026), rescinding the 2011 guidance. The 2026 definition is narrower — a 'complex' quantitative method applying statistical, economic or financial theories, expressly excluding simple arithmetic such as spreadsheet calculations and deterministic rule-based processes, and expressly excluding generative and agentic AI. CPS XXXX does not adopt that narrowing, for the reasons given in the standard. The divergence is deliberate.</t>
   </si>
   <si>
     <t xml:space="preserve">The definition is function-based. Whether the processing component is a linear regression, a deterministic actuarial projection, a decision tree, a gradient-boosted ensemble or a large language model does not change whether the tool is a model. Defining scope by technology creates a perimeter that moves every time the technology does.</t>
@@ -4413,7 +4413,7 @@
     <t xml:space="preserve">The accountable executive should be positioned to require change. Accountability without the authority to direct remediation, or without independence from the businesses whose models are being governed, is unlikely to be effective.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verification: the PRA allocates model risk management framework accountability to a designated senior management function. The precise interaction with the Australian accountability regime requires legal settlement and is flagged in Annex F of CPS 240.</t>
+    <t xml:space="preserve">Verification: the PRA allocates model risk management framework accountability to a designated senior management function. The precise interaction with the Australian accountability regime requires legal settlement and is flagged in Annex F of CPS XXXX.</t>
   </si>
   <si>
     <t xml:space="preserve">Each model should have a named owner accountable for it being fit for its approved purpose, for its documentation being current, for its performance being monitored, for its limitations being communicated to users, and for the remediation of findings. Ownership recorded in the inventory but not exercised is not ownership.</t>
@@ -4476,7 +4476,7 @@
     <t xml:space="preserve">Identification and inventory</t>
   </si>
   <si>
-    <t xml:space="preserve">The inventory is the foundation of the framework. No requirement in CPS 240 can be demonstrated for a model the entity does not know it has, and inventory completeness is therefore the first thing an entity should be able to evidence.</t>
+    <t xml:space="preserve">The inventory is the foundation of the framework. No requirement in CPS XXXX can be demonstrated for a model the entity does not know it has, and inventory completeness is therefore the first thing an entity should be able to evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: PRA SS1/23 Principle 1.2 Model inventory [SE]. OSFI Guideline E-23 (2027) Principle 2.1, on identifying and tracking all models in use or recently decommissioned [SE]. US interagency guidance 2026 §VI, model inventory [SE].</t>
@@ -4491,7 +4491,7 @@
     <t xml:space="preserve">The inventory should record decommissioned models where outputs they produced remain in force. A retired model that set a provision, a capital number, a customer price or an insurance liability that has not yet run off continues to carry model risk after the model itself has been switched off.</t>
   </si>
   <si>
-    <t xml:space="preserve">Annex B of CPS 240 sets out the minimum inventory fields. Entities should treat these as a floor. The inventory should be maintained as a controlled record with defined update responsibilities rather than as a periodically refreshed spreadsheet.</t>
+    <t xml:space="preserve">Annex B of CPS XXXX sets out the minimum inventory fields. Entities should treat these as a floor. The inventory should be maintained as a controlled record with defined update responsibilities rather than as a periodically refreshed spreadsheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Verification: inventory obligations were confirmed from the primary text of the PRA, OSFI and US instruments. OSFI's express inclusion of recently decommissioned models is extracted from Principle 2.1 of Guideline E-23 (2027).</t>
@@ -4716,7 +4716,7 @@
     <t xml:space="preserve">Source: CPS 230 Operational Risk Management, service provider management [B]. BCBS Principles for the sound management of third-party risk [B where implemented].</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 does not require access to vendor source code or training data. It requires sufficient information, or sufficient compensating control, for the entity to form a view on fitness for its own use.</t>
+    <t xml:space="preserve">CPS XXXX does not require access to vendor source code or training data. It requires sufficient information, or sufficient compensating control, for the entity to form a view on fitness for its own use.</t>
   </si>
   <si>
     <t xml:space="preserve">Concentration should be assessed at entity level and, so far as observable, across the industry. Widespread reliance on the same external model, data source or platform can produce correlated error across firms even where each firm's own governance is sound, and this is a supervisory concern that no individual firm's controls address.</t>
@@ -4728,7 +4728,7 @@
     <t xml:space="preserve">Artificial intelligence and machine learning models</t>
   </si>
   <si>
-    <t xml:space="preserve">An artificial intelligence or machine learning model is a model. Every requirement of CPS 240 applies to it. This chapter addresses the respects in which those requirements are harder to satisfy, not a separate regime.</t>
+    <t xml:space="preserve">An artificial intelligence or machine learning model is a model. Every requirement of CPS XXXX applies to it. This chapter addresses the respects in which those requirements are harder to satisfy, not a separate regime.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: OSFI Guideline E-23 (2027), which expressly brings AI and machine learning models within model risk management [SE]. MAS, Artificial Intelligence Model Risk Management information paper [G]. BCBS, Digitalisation of finance [A].</t>
@@ -4755,7 +4755,7 @@
     <t xml:space="preserve">Retraining should be monitored for stability. A model whose behaviour changes materially between retraining cycles on similar data is exhibiting a form of instability that periodic validation will not detect.</t>
   </si>
   <si>
-    <t xml:space="preserve">Where an entity operates a separate AI risk management framework, the two address different risks in the same system. CPS 240 governs whether a quantitative output is fit to be relied upon. AI risk management governs the wider consequences of the system's operation, including security, autonomy, data handling, human oversight and resilience.</t>
+    <t xml:space="preserve">Where an entity operates a separate AI risk management framework, the two address different risks in the same system. CPS XXXX governs whether a quantitative output is fit to be relied upon. AI risk management governs the wider consequences of the system's operation, including security, autonomy, data handling, human oversight and resilience.</t>
   </si>
   <si>
     <t xml:space="preserve">A generative or agentic system that produces no quantitative estimate used in decision-making is generally not a model, but remains subject to the entity's AI risk arrangements. A generative system used to produce an estimate that drives a material decision falls within both.</t>
@@ -4764,13 +4764,13 @@
     <t xml:space="preserve">The entity should record, for each AI system, which framework or frameworks apply, so that the boundary is a documented determination that can be reviewed rather than an assumption that can leave a system ungoverned.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verification: no comparator authority operates parallel model risk and AI risk instruments; OSFI deliberately brought AI within a single model risk guideline. The boundary rule in CPS 240 is therefore an Australian drafting choice arising from the proposed two-instrument architecture, and is identified as a policy design choice requiring consultation.</t>
+    <t xml:space="preserve">Verification: no comparator authority operates parallel model risk and AI risk instruments; OSFI deliberately brought AI within a single model risk guideline. The boundary rule in CPS XXXX is therefore an Australian drafting choice arising from the proposed two-instrument architecture, and is identified as a policy design choice requiring consultation.</t>
   </si>
   <si>
     <t xml:space="preserve">Specialist model classes</t>
   </si>
   <si>
-    <t xml:space="preserve">Models used to determine a regulatory capital requirement remain subject to the approval and change requirements of the applicable capital standard. CPS 240 sits alongside those requirements and does not displace them; where the two overlap, the more specific requirement prevails.</t>
+    <t xml:space="preserve">Models used to determine a regulatory capital requirement remain subject to the approval and change requirements of the applicable capital standard. CPS XXXX sits alongside those requirements and does not displace them; where the two overlap, the more specific requirement prevails.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: APS 113 Capital Adequacy: Internal Ratings-based Approach to Credit Risk [B]. ECB Guide to internal models [SE], interpreting binding Capital Requirements Regulation provisions [B]. PRA SS1/23, which applies to firms with internal model approval [SE].</t>
@@ -4791,7 +4791,7 @@
     <t xml:space="preserve">For an insurer, the Appointed Actuary framework already provides a form of independent professional review that will discharge a substantial part of the validation expectation for many actuarial models. It does not automatically discharge all of it, particularly implementation verification and data quality assessment.</t>
   </si>
   <si>
-    <t xml:space="preserve">Insurers should map which elements of CPS 240 validation are met through the actuarial control cycle and which require separate work, rather than assuming complete overlap in either direction. The mapping should be documented and reviewed.</t>
+    <t xml:space="preserve">Insurers should map which elements of CPS XXXX validation are met through the actuarial control cycle and which require separate work, rather than assuming complete overlap in either direction. The mapping should be documented and reviewed.</t>
   </si>
   <si>
     <t xml:space="preserve">Verification: OSFI's extension of Guideline E-23 (2027) to life and property and casualty insurers establishes the precedent for applying model risk management to insurance models. The specific interaction with the Australian Appointed Actuary framework is an Australian drafting question flagged for legal settlement.</t>
@@ -4848,7 +4848,7 @@
     <t xml:space="preserve">Early engagement is expected where an entity identifies a material weakness in a model used for regulatory capital, reserving or reporting. Engagement at the point the correction is finalised gives APRA no opportunity to consider the issue while options remain open.</t>
   </si>
   <si>
-    <t xml:space="preserve">Where a model failure is also an operational risk or information security incident, the notification requirements of the applicable prudential standards apply. CPS 240 does not create a separate or conflicting deadline.</t>
+    <t xml:space="preserve">Where a model failure is also an operational risk or information security incident, the notification requirements of the applicable prudential standards apply. CPS XXXX does not create a separate or conflicting deadline.</t>
   </si>
   <si>
     <t xml:space="preserve">Verification: the decision not to introduce a model-risk-specific notification deadline was deliberate. Introducing one risked conflicting with existing materiality criteria and timeframes, and is recorded as a correction in the red-team audit trail.</t>
@@ -4857,7 +4857,7 @@
     <t xml:space="preserve">Implementation</t>
   </si>
   <si>
-    <t xml:space="preserve">APRA recognises that meeting CPS 240 will require material uplift for many entities, particularly in inventory completeness, tiering consistency and validation coverage. The following phasing is indicative and would be settled through consultation.</t>
+    <t xml:space="preserve">APRA recognises that meeting CPS XXXX will require material uplift for many entities, particularly in inventory completeness, tiering consistency and validation coverage. The following phasing is indicative and would be settled through consultation.</t>
   </si>
   <si>
     <t xml:space="preserve">Entities should sequence by risk rather than by convenience. Establishing validation for the highest-tier models before completing the inventory of the lowest is generally the better order, provided discovery continues in parallel.</t>
@@ -5754,7 +5754,7 @@
     <t xml:space="preserve">ST-01</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 / CPG 240</t>
+    <t xml:space="preserve">CPS XXXX / CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">US legal status</t>
@@ -5790,13 +5790,13 @@
     <t xml:space="preserve">ST-03</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 M02</t>
+    <t xml:space="preserve">CPS XXXX M02</t>
   </si>
   <si>
     <t xml:space="preserve">US model definition</t>
   </si>
   <si>
-    <t xml:space="preserve">The current US definition is narrower than the definition adopted in CPS 240 and excludes spreadsheet arithmetic, deterministic rule-based processes, and generative and agentic AI.</t>
+    <t xml:space="preserve">The current US definition is narrower than the definition adopted in CPS XXXX and excludes spreadsheet arithmetic, deterministic rule-based processes, and generative and agentic AI.</t>
   </si>
   <si>
     <t xml:space="preserve">SR 26-2 §II and footnote 3.</t>
@@ -5808,7 +5808,7 @@
     <t xml:space="preserve">ST-04</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 M22 / CPG 240</t>
+    <t xml:space="preserve">CPS XXXX M22 / CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Effective challenge survives in the 2026 US guidance, reformulated around expertise, sufficient independence, and organisational standing and influence to effect change.</t>
@@ -5823,7 +5823,7 @@
     <t xml:space="preserve">ST-05</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 M21 / CPG 240</t>
+    <t xml:space="preserve">CPS XXXX M21 / CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">The components of validation are conceptual soundness, outcomes analysis and ongoing model monitoring.</t>
@@ -5895,7 +5895,7 @@
     <t xml:space="preserve">ST-10</t>
   </si>
   <si>
-    <t xml:space="preserve">CPG 240 Annex</t>
+    <t xml:space="preserve">CPG XXXX Annex</t>
   </si>
   <si>
     <t xml:space="preserve">CRR binding articles</t>
@@ -5937,7 +5937,7 @@
     <t xml:space="preserve">ST-13</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 M38 / CPG 240</t>
+    <t xml:space="preserve">CPS XXXX M38 / CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Superannuation</t>
@@ -5955,7 +5955,7 @@
     <t xml:space="preserve">ST-14</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240 M43 / CPG 240</t>
+    <t xml:space="preserve">CPS XXXX M43 / CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Notification</t>
@@ -5973,7 +5973,7 @@
     <t xml:space="preserve">ST-15</t>
   </si>
   <si>
-    <t xml:space="preserve">CPG 240</t>
+    <t xml:space="preserve">CPG XXXX</t>
   </si>
   <si>
     <t xml:space="preserve">Community bank proportionality</t>
@@ -6054,13 +6054,13 @@
     <t xml:space="preserve">RT-02</t>
   </si>
   <si>
-    <t xml:space="preserve">CPS 240's model definition was presented as following the established three-part US formulation, implying current US support for a broad definition.</t>
+    <t xml:space="preserve">CPS XXXX's model definition was presented as following the established three-part US formulation, implying current US support for a broad definition.</t>
   </si>
   <si>
     <t xml:space="preserve">Does the current US guidance still support a broad definition? If not, the standard is claiming alignment it does not have.</t>
   </si>
   <si>
-    <t xml:space="preserve">The 2026 US guidance narrows the definition to a 'complex' quantitative method applying statistical, economic or financial theories and expressly excludes simple arithmetic such as spreadsheet calculations, deterministic rule-based processes, and generative and agentic AI. CPS 240 retains the broad definition — deliberately, because the narrow one would exclude actuarial and unit pricing calculations central to the Australian cross-industry perimeter — and the divergence is now stated openly rather than concealed by a citation.</t>
+    <t xml:space="preserve">The 2026 US guidance narrows the definition to a 'complex' quantitative method applying statistical, economic or financial theories and expressly excludes simple arithmetic such as spreadsheet calculations, deterministic rule-based processes, and generative and agentic AI. CPS XXXX retains the broad definition — deliberately, because the narrow one would exclude actuarial and unit pricing calculations central to the Australian cross-industry perimeter — and the divergence is now stated openly rather than concealed by a citation.</t>
   </si>
   <si>
     <t xml:space="preserve">M02 rewritten; its provenance changed from Extracted to Extracted + inferred; the benchmark authority for the definition domain moved from the US to the PRA and OSFI.</t>

</xml_diff>

<commit_message>
Apply red-team operability corrections
Adds the missing APRA front matter (A1-A6: authority, application,
commencement, transition for models already in use, adjustments and
exclusions, interpretation) without which the instrument had no lawful
route to vary a requirement and would have prohibited continued use of
existing models on commencement.

Nine further corrections: M04 no longer lets an entity except itself
from mandatory requirements; M21 no longer demands outcomes analysis
where no outcome is observable; M20 gains an urgent-business-need path;
M40 works for RSE licensees, which have no internal capital assessment;
M13, M31, M32 and M37 made achievable; M43 and M03 made testable; and
the guide's validation table states drivers rather than intervals.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9tVmgcRH2aPufRoj4ddoe
</commit_message>
<xml_diff>
--- a/MRM_Regulatory_Comparison_and_Improvement_Assessment.xlsx
+++ b/MRM_Regulatory_Comparison_and_Improvement_Assessment.xlsx
@@ -952,7 +952,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4133" uniqueCount="1960">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4205" uniqueCount="2014">
   <si>
     <t xml:space="preserve">Model risk management package — workbook guide</t>
   </si>
@@ -3357,7 +3357,7 @@
     <t xml:space="preserve">Quantitative tools that are not models</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must identify material quantitative decision tools that fall outside its model definition, record them, and apply controls proportionate to the risk they present.</t>
+    <t xml:space="preserve">An APRA-regulated entity must identify material quantitative decision tools that fall outside its model definition — being tools whose output is fully determined by their inputs and documented rules, without estimation, statistical inference or an embedded assumption about an uncertain quantity — record them, and apply controls proportionate to the risk they present.</t>
   </si>
   <si>
     <t xml:space="preserve">The PRA expressly requires firms to consider quantitative methods that fall outside the model definition; without this, a narrow model definition becomes a control gap.</t>
@@ -3378,7 +3378,7 @@
     <t xml:space="preserve">Proportionality and controlled exceptions</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must apply this Prudential Standard in a manner proportionate to the materiality, complexity, autonomy and criticality of each model and to the size and business mix of the entity, and must document, time-bound, approve at an authority commensurate with the risk, and periodically review any exception to or reduction of the controls otherwise required.</t>
+    <t xml:space="preserve">An APRA-regulated entity must apply this Prudential Standard in a manner proportionate to the materiality, complexity, autonomy and criticality of each model and to the size and business mix of the entity, must be able to demonstrate that the intensity of controls applied to each model reflects its model risk tier and that models of equivalent tier are treated consistently, and must document, time-bound, approve at an authority commensurate with the risk and periodically review any departure from its own model risk policies and standards.</t>
   </si>
   <si>
     <t xml:space="preserve">PRA-SS1-23, OSFI-E23, US-MRM-2026, APRA-CPS220, BCBS-239</t>
@@ -3576,7 +3576,7 @@
     <t xml:space="preserve">Model identification and enterprise inventory</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must maintain a complete, accurate and current enterprise-wide inventory of its models, including models supplied by third parties, models embedded in acquired systems, models under development and models that have been retired but whose outputs remain in use.</t>
+    <t xml:space="preserve">An APRA-regulated entity must maintain an enterprise-wide inventory of its models and must maintain processes designed to ensure that the inventory is complete, accurate and current, including models supplied by third parties, models embedded in acquired systems, models under development and models that have been retired but whose outputs remain in use.</t>
   </si>
   <si>
     <t xml:space="preserve">PRA-SS1-23, US-MRM-2026, OSFI-E23, ECB-GIM, MAS-AIMRM-2024</t>
@@ -3723,7 +3723,7 @@
     <t xml:space="preserve">13. Independent validation</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must subject each model to independent validation before it is used for a material purpose and periodically thereafter at a frequency determined by its tier, and must not treat validation performed by the model's developer, its business sponsor or its vendor as satisfying this requirement.</t>
+    <t xml:space="preserve">An APRA-regulated entity must subject each model to independent validation before it is used for a material purpose and periodically thereafter at a frequency determined by its tier, and must not treat validation performed by the model's developer, its business sponsor or its vendor as satisfying this requirement. Where an urgent business need requires a model to be used before independent validation is complete, the entity must approve that use at an authority commensurate with the model's tier, apply compensating controls, inform users of the limitation and complete the validation within a defined period.</t>
   </si>
   <si>
     <t xml:space="preserve">US-MRM-2026, PRA-SS1-23, OSFI-E23, ECB-GIM, MAS-NOTICE637</t>
@@ -3744,7 +3744,7 @@
     <t xml:space="preserve">Scope of validation</t>
   </si>
   <si>
-    <t xml:space="preserve">Validation of a model must address conceptual soundness, outcomes analysis comparing model outputs with corresponding actual outcomes, and ongoing model monitoring, and must reach an explicit conclusion on the model's fitness for its intended use together with any conditions or limitations.</t>
+    <t xml:space="preserve">Validation of a model must address conceptual soundness, ongoing model monitoring, and outcomes analysis comparing model outputs with corresponding actual outcomes to the extent those outcomes are observable and sufficient for the purpose, and must reach an explicit conclusion on the model's fitness for its intended use together with any conditions or limitations. Where outcomes are not observable, the entity must apply alternative evidence of performance, including benchmarking, sensitivity analysis and assessment of assumptions.</t>
   </si>
   <si>
     <t xml:space="preserve">The three core elements of validation are the most widely adopted formulation in the discipline and originate in the US interagency guidance.</t>
@@ -3924,7 +3924,7 @@
     <t xml:space="preserve">Vendor and externally developed models</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must apply this Prudential Standard to models supplied, hosted or operated by third parties, and must obtain information sufficient to understand the model's design, data, assumptions, limitations and performance, or implement compensating controls where that information cannot be obtained.</t>
+    <t xml:space="preserve">An APRA-regulated entity must apply this Prudential Standard to models supplied, hosted or operated by third parties, and must obtain information sufficient to understand the model's design, data, assumptions, limitations and performance. Where the entity cannot itself discharge an obligation in this Prudential Standard in relation to a third-party model, it must obtain equivalent assurance from the provider or implement compensating controls, and must record which obligations are met in that way.</t>
   </si>
   <si>
     <t xml:space="preserve">US-MRM-2026, OSFI-E23, BCBS-TPRM, APRA-CPS230, PRA-SS1-23</t>
@@ -3942,7 +3942,7 @@
     <t xml:space="preserve">Information rights, concentration and substitutability</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must maintain contractual and governance arrangements giving it timely access to the information and assurance it needs to meet its obligations in relation to a material third-party model, and must identify and manage concentration and substitutability risk arising from common models, data sources, platforms and providers.</t>
+    <t xml:space="preserve">An APRA-regulated entity must maintain contractual and governance arrangements giving it timely access to the information and assurance it needs to meet its obligations in relation to a material third-party model, and must identify and manage concentration and substitutability risk arising from common models, data sources, platforms and providers. Where an arrangement is already on foot at the commencement of this Prudential Standard, this paragraph applies from the earlier of the next renewal or material variation of that arrangement and the end of the transition period determined by APRA.</t>
   </si>
   <si>
     <t xml:space="preserve">APRA-CPS230, BCBS-TPRM, FSB-AI-2024, OSFI-E23</t>
@@ -4053,7 +4053,7 @@
     <t xml:space="preserve">Actuarial, reserving and insurance liability models</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated insurer must apply this Prudential Standard to models used to determine insurance liabilities, premiums, reinsurance recoveries and capital, and must ensure that the role of the Appointed Actuary and this Prudential Standard's validation requirements operate together without gaps in independent review.</t>
+    <t xml:space="preserve">An APRA-regulated insurer must apply this Prudential Standard to models used to determine insurance liabilities, premiums, reinsurance recoveries and capital, and must ensure that the role of the Appointed Actuary and this Prudential Standard's validation requirements operate together without gaps in independent review. Independent review performed under CPS 320 and the sectoral actuarial standards may satisfy the independent validation requirement for an actuarial model to the extent the reviewer was not responsible for developing the model or setting its assumptions, and the insurer must identify and separately address any element not so covered.</t>
   </si>
   <si>
     <t xml:space="preserve">APRA-CPS320, APRA-GPS320, APRA-LPS320, OSFI-E23</t>
@@ -4122,7 +4122,7 @@
     <t xml:space="preserve">Aggregate assessment of model risk</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must assess model risk in aggregate across its model portfolio, must consider the effect of that aggregate risk in its internal capital assessment, and must be able to explain the basis and limitations of the assessment.</t>
+    <t xml:space="preserve">An APRA-regulated entity must assess model risk in aggregate across its model portfolio, must consider the effect of that aggregate risk in its internal capital adequacy assessment or, for an RSE licensee, in determining its operational risk financial requirement target amount, and must be able to explain the basis and limitations of the assessment.</t>
   </si>
   <si>
     <t xml:space="preserve">PRA-SS1-23, ECB-GIM, US-MRM-2026, APRA-CPS220</t>
@@ -4179,7 +4179,7 @@
     <t xml:space="preserve">Notification and provision of information to APRA</t>
   </si>
   <si>
-    <t xml:space="preserve">An APRA-regulated entity must notify APRA of a model failure or model risk event that has, or is likely to have, a material impact on its financial position, its regulatory reporting or its ability to meet its prudential obligations, and must provide APRA with information relating to its models and model risk management on request.</t>
+    <t xml:space="preserve">An APRA-regulated entity must notify APRA as soon as practicable, and within the timeframe applicable under CPS 230 or CPS 234 where the event also falls within those standards, of a model failure or model risk event that has, or is likely to have, a material impact on its financial position, its regulatory reporting or its ability to meet its prudential obligations, and must provide APRA with information relating to its models and model risk management on request.</t>
   </si>
   <si>
     <t xml:space="preserve">APRA-CPS230, APRA-CPS234, APRA-CPS220, OSFI-E23</t>
@@ -4599,7 +4599,7 @@
     <t xml:space="preserve">A validation report should reach an explicit conclusion on fitness for the intended use, with any conditions or limitations stated. A report that records observations without a conclusion leaves the approval decision without the input it was designed to receive.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verification: the three core elements of validation are extracted from the US interagency guidance, which remains supervisory guidance rather than a regulation. Validation frequencies in the table above are illustrative drafting and are not taken from any comparator instrument; they are identified as a policy design choice in the assessment workbook.</t>
+    <t xml:space="preserve">Verification: the three components of validation are extracted from the current US interagency guidance, which is supervisory guidance rather than a regulation and is non-enforceable by its own terms. No fixed validation frequency is stated in this guide: the rescinded 2011 US guidance contained an at-least-annual periodic review expectation which the April 2026 guidance does not carry forward, and OCC Bulletin 2025-26 confirms that community banks are not required to validate annually. Setting cycle lengths is left to the entity, by tier.</t>
   </si>
   <si>
     <t xml:space="preserve">Effective challenge is critical and objective analysis by people with three attributes together: the expertise to identify model limitations, sufficient independence to maintain objectivity, and the organisational standing and influence to bring about change. Removing any one defeats the control while leaving its documentation intact. Entities should also attend to incentives, since a challenger rewarded for clearing models will not challenge for long.</t>
@@ -6496,6 +6496,168 @@
   </si>
   <si>
     <t xml:space="preserve">Closed — limitation disclosed rather than concealed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The standard opened at 'Objectives and key requirements' with no Authority, Application, Commencement or Adjustments and exclusions paragraphs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every APRA prudential standard carries this front matter. Without an adjustments and exclusions paragraph there is no lawful route for APRA to vary a requirement for an individual entity, making the instrument more rigid than every standard it sits alongside. Without a transitional paragraph, requirements expressed as a bar on use would on commencement prohibit continued use of models entities already rely on.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paragraphs A1 to A6 were added: authority, application, commencement, transitional arrangements for models already in use, adjustments and exclusions, and interpretation. Each carries a note identifying what requires legal settlement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Six new mandatory paragraphs; the standard is now structurally complete as an instrument.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPS 230 paragraphs 1 to 11 as the structural precedent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M04 required an entity to document and approve 'any exception to or reduction of the controls otherwise required' by the standard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The controls otherwise required are the mandatory paragraphs. As drafted, a proportionality clause purported to let an entity except itself from the instrument's own requirements at its own approval authority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M04 was split in substance: it now requires the entity to demonstrate that control intensity reflects the model's tier and that equivalent models are treated consistently, and confines the exception machinery to departures from the entity's own policies and standards. The guidance states plainly that only APRA may adjust or exclude a requirement, under A5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M04 redrafted; its guidance rewritten; the adjustment power now sits in A5 where it belongs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal analysis of the interaction between M04 and the mandatory paragraphs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M21 required validation to address outcomes analysis comparing model outputs with corresponding actual outcomes, without qualification.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For several model classes the standard expressly brings into scope — stress testing, scenario analysis, capital planning and forward-looking climate models — no corresponding actual outcome exists. The requirement was impossible to satisfy for them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M21 now requires outcomes analysis to the extent outcomes are observable and sufficient for the purpose, and requires alternative evidence of performance — benchmarking, sensitivity analysis and assessment of assumptions — where they are not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M21 redrafted; the validation intensity table in the guide realigned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M39 scope; BCBS stress testing principles 7 and 8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M20 barred use of a model for a material purpose until independent validation was complete, with no exception path.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The current US guidance expressly contemplates use before validation on urgent business need with compensating controls. An absolute bar with no exception and no transition would on commencement prohibit continued use of every insufficiently validated model in the industry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M20 now permits use before validation completes where there is an urgent business need, subject to approval at an authority commensurate with tier, compensating controls, informing users of the limitation and completing validation within a defined period. Paragraph A4 provides the transition for models already in use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M20 redrafted; A4 added.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US interagency guidance 2026 §V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M40 required every APRA-regulated entity to consider aggregate model risk in its internal capital assessment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSE licensees have no internal capital assessment. The requirement was inapplicable to an entire regulated industry the standard purports to cover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M40 now refers to the internal capital adequacy assessment or, for an RSE licensee, to determining the operational risk financial requirement target amount.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M40 redrafted sector-neutrally.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superannuation prudential framework; SPS 114 operational risk financial requirement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M13 required a complete, accurate and current inventory in absolute terms; M31's compensating-control escape reached only the information limb; M32 had no transition for contracts already on foot; and M37 left the Appointed Actuary conflict to the guide.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Absolute completeness is not demonstrable and not testable. A hosted vendor model cannot be subjected to the entity's own implementation controls. Existing contracts cannot be reopened on commencement. And for most insurers the Appointed Actuary sets the assumptions, so M08 and M20 would disqualify the very review CPS 320 requires.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M13 now requires the inventory plus processes designed to ensure completeness. M31's escape extends to any obligation the entity cannot itself discharge for a third-party model, with a record of which are met that way. M32 applies to existing arrangements from the earlier of renewal, material variation or the end of the transition period. M37 resolves the actuarial interaction in the standard: CPS 320 review satisfies independent validation to the extent the reviewer did not develop the model or set its assumptions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four requirements redrafted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPS 230 transitional precedent for service provider arrangements; CPS 320.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The practice guide's validation intensity table prescribed 'at least annually' for the highest tier and 'every two to three years' for the second, while its own caption called the frequencies illustrative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A table that states an interval will be read as the expectation whatever the caption says. No comparator prescribes cross-industry validation frequencies, and the OCC has expressly confirmed that its guidance does not require annual validation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The frequency cells now state the drivers rather than intervals, and the caption and verification note explain why no interval is given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chapter 8 of the practice guide.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCC Bulletin 2025-26; US interagency guidance 2026 §V; PRA SS1/23 Principle 4.5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M43 created a notification obligation with no timeframe and no threshold beyond 'material', while the guidance beneath it told entities to use CPS 230 and CPS 234 timeframes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The requirement and its guidance said different things, and the requirement as drafted was not testable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M43 now states the timing expectation on the face of the requirement and ties it to the CPS 230 and CPS 234 timeframes where the event falls within those standards, resolving the inconsistency without creating a competing deadline.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M43 redrafted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPS 230; CPS 234.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M03 identified non-model quantitative tools by example only — spreadsheets, rules engines, allocation keys — with no stated criterion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples cannot draw a perimeter. A complex spreadsheet running a regression is a model; a complex spreadsheet applying documented arithmetic is not. The examples invited the wrong reading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M03 now states the criterion on the face of the requirement: a tool falls outside the model definition only where its output is fully determined by its inputs and documented rules, without estimation, statistical inference or an embedded assumption about an uncertain quantity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M03 redrafted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRA SS1/23 Principle 1.1; US interagency guidance 2026 §II exclusions.</t>
   </si>
   <si>
     <t xml:space="preserve">RT-18</t>
@@ -13005,7 +13167,7 @@
     <tabColor rgb="FF1B335F"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -13697,15 +13859,249 @@
         <v>1853</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>1706</v>
       </c>
     </row>
+    <row r="30" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>1854</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>1856</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>1857</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>1858</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>1859</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>1860</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>1862</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>1863</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>1864</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>1865</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>1866</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>1867</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>1868</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>1869</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>1870</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>1871</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>1872</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1873</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>1874</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>1875</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>1876</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>1877</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>1879</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>1880</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>1881</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>1882</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>1883</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>1884</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>1885</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>1886</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>1887</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>1888</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>1889</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>1890</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>1891</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>1892</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>1893</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>1894</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>1895</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>1896</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>1897</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>1898</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>1899</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>1900</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>1901</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>1902</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>1903</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>1904</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>1905</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>1906</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>1907</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>1706</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:H4"/>
-  <conditionalFormatting sqref="G5:G29">
+  <conditionalFormatting sqref="G5:G38">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"REFUTED"</formula>
     </cfRule>
@@ -13761,12 +14157,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1854</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1855</v>
+        <v>1909</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13789,16 +14185,16 @@
         <v>585</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>1856</v>
+        <v>1910</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1857</v>
+        <v>1911</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>587</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>1858</v>
+        <v>1912</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13821,16 +14217,16 @@
         <v>592</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>1859</v>
+        <v>1913</v>
       </c>
       <c r="H5" s="24" t="s">
-        <v>1860</v>
+        <v>1914</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13853,16 +14249,16 @@
         <v>600</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>1862</v>
+        <v>1916</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>1863</v>
+        <v>1917</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13885,16 +14281,16 @@
         <v>606</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>1864</v>
+        <v>1918</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>1865</v>
+        <v>1919</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13917,16 +14313,16 @@
         <v>613</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>1866</v>
+        <v>1920</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>1867</v>
+        <v>1921</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13949,16 +14345,16 @@
         <v>619</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>1868</v>
+        <v>1922</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>1869</v>
+        <v>1923</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>621</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13981,16 +14377,16 @@
         <v>626</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>1870</v>
+        <v>1924</v>
       </c>
       <c r="H10" s="25" t="s">
-        <v>1871</v>
+        <v>1925</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14013,16 +14409,16 @@
         <v>631</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>1872</v>
+        <v>1926</v>
       </c>
       <c r="H11" s="24" t="s">
-        <v>1871</v>
+        <v>1925</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14045,16 +14441,16 @@
         <v>637</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>1873</v>
+        <v>1927</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>1874</v>
+        <v>1928</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14077,16 +14473,16 @@
         <v>643</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>1875</v>
+        <v>1929</v>
       </c>
       <c r="H13" s="24" t="s">
-        <v>1876</v>
+        <v>1930</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14109,16 +14505,16 @@
         <v>648</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>1877</v>
+        <v>1931</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>1878</v>
+        <v>1932</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14141,16 +14537,16 @@
         <v>654</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>1879</v>
+        <v>1933</v>
       </c>
       <c r="H15" s="24" t="s">
-        <v>1880</v>
+        <v>1934</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14173,16 +14569,16 @@
         <v>660</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>1881</v>
+        <v>1935</v>
       </c>
       <c r="H16" s="25" t="s">
-        <v>1882</v>
+        <v>1936</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14205,16 +14601,16 @@
         <v>666</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>1883</v>
+        <v>1937</v>
       </c>
       <c r="H17" s="24" t="s">
-        <v>1884</v>
+        <v>1938</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14237,16 +14633,16 @@
         <v>671</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>1885</v>
+        <v>1939</v>
       </c>
       <c r="H18" s="25" t="s">
-        <v>1886</v>
+        <v>1940</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14269,16 +14665,16 @@
         <v>677</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>1887</v>
+        <v>1941</v>
       </c>
       <c r="H19" s="24" t="s">
-        <v>1888</v>
+        <v>1942</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14301,16 +14697,16 @@
         <v>682</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>1889</v>
+        <v>1943</v>
       </c>
       <c r="H20" s="25" t="s">
-        <v>1890</v>
+        <v>1944</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14333,16 +14729,16 @@
         <v>687</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>1891</v>
+        <v>1945</v>
       </c>
       <c r="H21" s="24" t="s">
-        <v>1892</v>
+        <v>1946</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14365,16 +14761,16 @@
         <v>693</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>1893</v>
+        <v>1947</v>
       </c>
       <c r="H22" s="25" t="s">
-        <v>1894</v>
+        <v>1948</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14397,16 +14793,16 @@
         <v>698</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>1895</v>
+        <v>1949</v>
       </c>
       <c r="H23" s="24" t="s">
-        <v>1896</v>
+        <v>1950</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14429,16 +14825,16 @@
         <v>703</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>1897</v>
+        <v>1951</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>1898</v>
+        <v>1952</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14461,16 +14857,16 @@
         <v>708</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>1899</v>
+        <v>1953</v>
       </c>
       <c r="H25" s="24" t="s">
-        <v>1900</v>
+        <v>1954</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14493,16 +14889,16 @@
         <v>712</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>1901</v>
+        <v>1955</v>
       </c>
       <c r="H26" s="25" t="s">
-        <v>1902</v>
+        <v>1956</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14525,16 +14921,16 @@
         <v>716</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>1903</v>
+        <v>1957</v>
       </c>
       <c r="H27" s="24" t="s">
-        <v>1904</v>
+        <v>1958</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14557,16 +14953,16 @@
         <v>721</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>1905</v>
+        <v>1959</v>
       </c>
       <c r="H28" s="25" t="s">
-        <v>1906</v>
+        <v>1960</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14589,16 +14985,16 @@
         <v>726</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>1907</v>
+        <v>1961</v>
       </c>
       <c r="H29" s="24" t="s">
-        <v>1908</v>
+        <v>1962</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14621,16 +15017,16 @@
         <v>732</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>1909</v>
+        <v>1963</v>
       </c>
       <c r="H30" s="25" t="s">
-        <v>1910</v>
+        <v>1964</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14653,16 +15049,16 @@
         <v>738</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>1911</v>
+        <v>1965</v>
       </c>
       <c r="H31" s="24" t="s">
-        <v>1912</v>
+        <v>1966</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14685,16 +15081,16 @@
         <v>744</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>1913</v>
+        <v>1967</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>1914</v>
+        <v>1968</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14717,16 +15113,16 @@
         <v>732</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>1915</v>
+        <v>1969</v>
       </c>
       <c r="H33" s="24" t="s">
-        <v>1916</v>
+        <v>1970</v>
       </c>
       <c r="I33" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14749,16 +15145,16 @@
         <v>752</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>1917</v>
+        <v>1971</v>
       </c>
       <c r="H34" s="25" t="s">
-        <v>1918</v>
+        <v>1972</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14781,16 +15177,16 @@
         <v>738</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>1919</v>
+        <v>1973</v>
       </c>
       <c r="H35" s="24" t="s">
-        <v>1920</v>
+        <v>1974</v>
       </c>
       <c r="I35" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14813,16 +15209,16 @@
         <v>738</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>1921</v>
+        <v>1975</v>
       </c>
       <c r="H36" s="25" t="s">
-        <v>1922</v>
+        <v>1976</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14845,16 +15241,16 @@
         <v>738</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>1923</v>
+        <v>1977</v>
       </c>
       <c r="H37" s="24" t="s">
-        <v>1924</v>
+        <v>1978</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>594</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14877,16 +15273,16 @@
         <v>738</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>1925</v>
+        <v>1979</v>
       </c>
       <c r="H38" s="25" t="s">
-        <v>1926</v>
+        <v>1980</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>594</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>1861</v>
+        <v>1915</v>
       </c>
     </row>
   </sheetData>
@@ -14928,17 +15324,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1927</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1928</v>
+        <v>1982</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>1929</v>
+        <v>1983</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>75</v>
@@ -14946,42 +15342,42 @@
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>1930</v>
+        <v>1984</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>1931</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>1932</v>
+        <v>1986</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>1933</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>1934</v>
+        <v>1988</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>1935</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>1936</v>
+        <v>1990</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>1937</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>1938</v>
+        <v>1992</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>1939</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14989,7 +15385,7 @@
         <v>148</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>1940</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14997,47 +15393,47 @@
         <v>149</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>1941</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>1942</v>
+        <v>1996</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>1943</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>1944</v>
+        <v>1998</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>1945</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>1946</v>
+        <v>2000</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>1947</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>1948</v>
+        <v>2002</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1949</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>1950</v>
+        <v>2004</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>1951</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15045,7 +15441,7 @@
         <v>788</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>1952</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15053,7 +15449,7 @@
         <v>795</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>1953</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15061,7 +15457,7 @@
         <v>1042</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>1954</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15069,7 +15465,7 @@
         <v>1013</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>1955</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15077,7 +15473,7 @@
         <v>594</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>1956</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15085,15 +15481,15 @@
         <v>621</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>1957</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>1958</v>
+        <v>2012</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>1959</v>
+        <v>2013</v>
       </c>
     </row>
   </sheetData>
@@ -15258,7 +15654,7 @@
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">COUNTA('Red Team Audit'!A5:A200)</f>
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>50</v>
@@ -15270,7 +15666,7 @@
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">COUNTIF('Red Team Audit'!G5:G200,"High")</f>
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>52</v>

</xml_diff>